<commit_message>
Completed Basic Header Board for Power With Power Supply
</commit_message>
<xml_diff>
--- a/Legs Power Header/BOM.xlsx
+++ b/Legs Power Header/BOM.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Prints\Legs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\Prints\Legs\Legs Power Header\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{498BBA05-720D-42B4-AC58-CC0400D3BD3F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BF218634-ED12-4F6D-8426-A0D1FAF9618F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="18240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,12 +25,39 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>2223-SSK02-FPH-254-A4-ND</t>
   </si>
   <si>
     <t>1568-10474-ND</t>
+  </si>
+  <si>
+    <t>Item Number</t>
+  </si>
+  <si>
+    <t>Ref Des</t>
+  </si>
+  <si>
+    <t>J1</t>
+  </si>
+  <si>
+    <t>Quantity</t>
+  </si>
+  <si>
+    <t>Distributor Part Number</t>
+  </si>
+  <si>
+    <t>Manufacturer Part Number</t>
+  </si>
+  <si>
+    <t>Description</t>
+  </si>
+  <si>
+    <t>Unit Price</t>
+  </si>
+  <si>
+    <t>Total Cost</t>
   </si>
 </sst>
 </file>
@@ -66,8 +93,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -348,43 +378,76 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C3"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="12.85546875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.140625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A1">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C1" t="s">
+        <v>8</v>
+      </c>
+      <c r="D1" t="s">
+        <v>7</v>
+      </c>
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" t="s">
+        <v>9</v>
+      </c>
+      <c r="H1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2">
         <v>1</v>
       </c>
-      <c r="B1">
+      <c r="B2" t="s">
+        <v>4</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="F2">
         <v>12</v>
       </c>
-      <c r="C1" t="s">
-        <v>0</v>
-      </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3">
         <v>2</v>
       </c>
-      <c r="B2">
+      <c r="E3" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C2" t="s">
+      <c r="F3">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A4">
         <v>3</v>
       </c>
-      <c r="B3">
+      <c r="E4" s="1">
+        <v>1935776</v>
+      </c>
+      <c r="F4">
         <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1935776</v>
       </c>
     </row>
   </sheetData>

</xml_diff>